<commit_message>
Add SOH report for 2026-10-29
</commit_message>
<xml_diff>
--- a/reports/SOH_29_10_2026.xlsx
+++ b/reports/SOH_29_10_2026.xlsx
@@ -433,7 +433,7 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="D19" s="2" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>8856</v>
@@ -1478,7 +1478,7 @@
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>10735</v>
+        <v>10711</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>10251</v>
@@ -2094,7 +2094,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>6837</v>
@@ -3914,7 +3914,7 @@
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>311</v>
+        <v>287</v>
       </c>
       <c r="E124" s="3" t="n">
         <v>12281</v>
@@ -5006,7 +5006,7 @@
         </is>
       </c>
       <c r="D163" s="2" t="n">
-        <v>111</v>
+        <v>99</v>
       </c>
       <c r="E163" s="3" t="n">
         <v>8711</v>
@@ -8566,7 +8566,7 @@
         </is>
       </c>
       <c r="D293" s="2" t="n">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="E293" s="3" t="n">
         <v>0</v>
@@ -8766,7 +8766,7 @@
         </is>
       </c>
       <c r="D301" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E301" s="3" t="n">
         <v>1</v>
@@ -8822,7 +8822,7 @@
         </is>
       </c>
       <c r="D303" s="2" t="n">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E303" s="3" t="n">
         <v>1</v>
@@ -9046,7 +9046,7 @@
         </is>
       </c>
       <c r="D311" s="2" t="n">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E311" s="3" t="n">
         <v>1</v>
@@ -9074,7 +9074,7 @@
         </is>
       </c>
       <c r="D312" s="2" t="n">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="E312" s="3" t="n">
         <v>1</v>
@@ -9410,7 +9410,7 @@
         </is>
       </c>
       <c r="D324" s="2" t="n">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="E324" s="3" t="n">
         <v>1</v>
@@ -10138,7 +10138,7 @@
         </is>
       </c>
       <c r="D350" s="2" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E350" s="3" t="n">
         <v>20000</v>
@@ -10302,7 +10302,7 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Skincare Soap Strawberry (60*1Pc)</t>
+          <t>AIWIBI Baby Skincare Soap Strawberry</t>
         </is>
       </c>
       <c r="D356" s="2" t="n">
@@ -10442,7 +10442,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Strawberry) (96*1Pc)</t>
+          <t>AIWIBI Kid's Jolly Teeth Care Toothpaste(Strawberry)</t>
         </is>
       </c>
       <c r="D361" s="2" t="n">
@@ -10558,7 +10558,7 @@
         </is>
       </c>
       <c r="D365" s="2" t="n">
-        <v>574</v>
+        <v>555</v>
       </c>
       <c r="E365" s="3" t="n">
         <v>12500</v>
@@ -10586,7 +10586,7 @@
         </is>
       </c>
       <c r="D366" s="2" t="n">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="E366" s="3" t="n">
         <v>8000</v>
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="D373" s="2" t="n">
-        <v>1021</v>
+        <v>1012</v>
       </c>
       <c r="E373" s="3" t="n">
         <v>40000</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="D375" s="2" t="n">
-        <v>693</v>
+        <v>684</v>
       </c>
       <c r="E375" s="3" t="n">
         <v>40000</v>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
       <c r="D377" s="2" t="n">
-        <v>600</v>
+        <v>587</v>
       </c>
       <c r="E377" s="3" t="n">
         <v>40000</v>
@@ -10922,7 +10922,7 @@
         </is>
       </c>
       <c r="D378" s="2" t="n">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="E378" s="3" t="n">
         <v>10500</v>
@@ -10950,7 +10950,7 @@
         </is>
       </c>
       <c r="D379" s="2" t="n">
-        <v>297</v>
+        <v>282</v>
       </c>
       <c r="E379" s="3" t="n">
         <v>40000</v>
@@ -11286,7 +11286,7 @@
         </is>
       </c>
       <c r="D391" s="2" t="n">
-        <v>603</v>
+        <v>596</v>
       </c>
       <c r="E391" s="3" t="n">
         <v>51000</v>
@@ -11342,7 +11342,7 @@
         </is>
       </c>
       <c r="D393" s="2" t="n">
-        <v>932</v>
+        <v>921</v>
       </c>
       <c r="E393" s="3" t="n">
         <v>51000</v>
@@ -11398,7 +11398,7 @@
         </is>
       </c>
       <c r="D395" s="2" t="n">
-        <v>1277</v>
+        <v>1264</v>
       </c>
       <c r="E395" s="3" t="n">
         <v>51000</v>
@@ -11426,7 +11426,7 @@
         </is>
       </c>
       <c r="D396" s="2" t="n">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="E396" s="3" t="n">
         <v>26500</v>
@@ -11454,7 +11454,7 @@
         </is>
       </c>
       <c r="D397" s="2" t="n">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E397" s="3" t="n">
         <v>51000</v>
@@ -11482,7 +11482,7 @@
         </is>
       </c>
       <c r="D398" s="2" t="n">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E398" s="3" t="n">
         <v>26500</v>
@@ -11622,7 +11622,7 @@
         </is>
       </c>
       <c r="D403" s="2" t="n">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="E403" s="3" t="n">
         <v>81000</v>
@@ -11650,7 +11650,7 @@
         </is>
       </c>
       <c r="D404" s="2" t="n">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="E404" s="3" t="n">
         <v>81000</v>
@@ -11930,7 +11930,7 @@
         </is>
       </c>
       <c r="D414" s="2" t="n">
-        <v>2437</v>
+        <v>2417</v>
       </c>
       <c r="E414" s="3" t="n">
         <v>3876</v>
@@ -12014,7 +12014,7 @@
         </is>
       </c>
       <c r="D417" s="2" t="n">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E417" s="3" t="n">
         <v>8000</v>
@@ -12070,7 +12070,7 @@
         </is>
       </c>
       <c r="D419" s="2" t="n">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="E419" s="3" t="n">
         <v>10000</v>
@@ -12122,11 +12122,11 @@
       </c>
       <c r="C421" t="inlineStr">
         <is>
-          <t>AIWIBI Papaya Wet Wipes (4*3*84Pcs)</t>
+          <t>AIWIBI Baby Wet Wipes (4*3*84Pcs)</t>
         </is>
       </c>
       <c r="D421" s="2" t="n">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="E421" s="3" t="n">
         <v>21000</v>
@@ -12210,7 +12210,7 @@
         </is>
       </c>
       <c r="D424" s="2" t="n">
-        <v>-57</v>
+        <v>-58</v>
       </c>
       <c r="E424" s="3" t="n">
         <v>8000</v>
@@ -12714,7 +12714,7 @@
         </is>
       </c>
       <c r="D442" s="2" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E442" s="3" t="n">
         <v>3500</v>
@@ -12882,7 +12882,7 @@
         </is>
       </c>
       <c r="D448" s="2" t="n">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E448" s="3" t="n">
         <v>25000</v>
@@ -12910,7 +12910,7 @@
         </is>
       </c>
       <c r="D449" s="2" t="n">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E449" s="3" t="n">
         <v>25000</v>
@@ -12938,7 +12938,7 @@
         </is>
       </c>
       <c r="D450" s="2" t="n">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E450" s="3" t="n">
         <v>25000</v>
@@ -12966,7 +12966,7 @@
         </is>
       </c>
       <c r="D451" s="2" t="n">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="E451" s="3" t="n">
         <v>36000</v>
@@ -12994,7 +12994,7 @@
         </is>
       </c>
       <c r="D452" s="2" t="n">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E452" s="3" t="n">
         <v>36000</v>
@@ -13050,7 +13050,7 @@
         </is>
       </c>
       <c r="D454" s="2" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E454" s="3" t="n">
         <v>5000</v>
@@ -13106,7 +13106,7 @@
         </is>
       </c>
       <c r="D456" s="2" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E456" s="3" t="n">
         <v>5000</v>
@@ -13134,7 +13134,7 @@
         </is>
       </c>
       <c r="D457" s="2" t="n">
-        <v>1624</v>
+        <v>1612</v>
       </c>
       <c r="E457" s="3" t="n">
         <v>7090</v>
@@ -15122,7 +15122,7 @@
         </is>
       </c>
       <c r="D528" s="2" t="n">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="E528" s="3" t="n">
         <v>10733</v>
@@ -15430,7 +15430,7 @@
         </is>
       </c>
       <c r="D539" s="2" t="n">
-        <v>441</v>
+        <v>417</v>
       </c>
       <c r="E539" s="3" t="n">
         <v>9433</v>
@@ -15542,7 +15542,7 @@
         </is>
       </c>
       <c r="D543" s="2" t="n">
-        <v>934</v>
+        <v>922</v>
       </c>
       <c r="E543" s="3" t="n">
         <v>17750</v>
@@ -16074,7 +16074,7 @@
         </is>
       </c>
       <c r="D562" s="2" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E562" s="3" t="n">
         <v>12900</v>
@@ -16578,7 +16578,7 @@
         </is>
       </c>
       <c r="D580" s="2" t="n">
-        <v>1943</v>
+        <v>1937</v>
       </c>
       <c r="E580" s="3" t="n">
         <v>19364</v>
@@ -17110,7 +17110,7 @@
         </is>
       </c>
       <c r="D599" s="2" t="n">
-        <v>432</v>
+        <v>438</v>
       </c>
       <c r="E599" s="3" t="n">
         <v>10267</v>
@@ -17726,7 +17726,7 @@
         </is>
       </c>
       <c r="D621" s="2" t="n">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="E621" s="3" t="n">
         <v>13768</v>
@@ -18650,7 +18650,7 @@
         </is>
       </c>
       <c r="D654" s="2" t="n">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="E654" s="3" t="n">
         <v>14083</v>
@@ -18846,7 +18846,7 @@
         </is>
       </c>
       <c r="D661" s="2" t="n">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="E661" s="3" t="n">
         <v>25000</v>
@@ -18874,7 +18874,7 @@
         </is>
       </c>
       <c r="D662" s="2" t="n">
-        <v>369</v>
+        <v>362</v>
       </c>
       <c r="E662" s="3" t="n">
         <v>1</v>
@@ -20382,7 +20382,7 @@
       </c>
       <c r="C716" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Facial Cream (48*1Pc)</t>
+          <t>AIWIBI Baby Facial Cream</t>
         </is>
       </c>
       <c r="D716" s="2" t="n">
@@ -20414,7 +20414,7 @@
         </is>
       </c>
       <c r="D717" s="2" t="n">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="E717" s="3" t="n">
         <v>1</v>
@@ -23298,7 +23298,7 @@
         </is>
       </c>
       <c r="D820" s="2" t="n">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E820" s="3" t="n">
         <v>16983</v>
@@ -25590,11 +25590,11 @@
       </c>
       <c r="C902" t="inlineStr">
         <is>
-          <t>AWB Baby Laundry Detergent (1000ml) (12*1Pc)</t>
+          <t>AWB Baby Laundry Detergent (1000ml)</t>
         </is>
       </c>
       <c r="D902" s="2" t="n">
-        <v>613</v>
+        <v>606</v>
       </c>
       <c r="E902" s="3" t="n">
         <v>26000</v>
@@ -25622,7 +25622,7 @@
         </is>
       </c>
       <c r="D903" s="2" t="n">
-        <v>525</v>
+        <v>519</v>
       </c>
       <c r="E903" s="3" t="n">
         <v>4500</v>
@@ -25650,7 +25650,7 @@
         </is>
       </c>
       <c r="D904" s="2" t="n">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="E904" s="3" t="n">
         <v>1</v>
@@ -25930,7 +25930,7 @@
         </is>
       </c>
       <c r="D914" s="2" t="n">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E914" s="3" t="n">
         <v>20000</v>
@@ -25954,7 +25954,7 @@
       </c>
       <c r="C915" t="inlineStr">
         <is>
-          <t>AIWIBI Baby Mosquito Repellent Patches (96*1Pc)</t>
+          <t>AIWIBI Baby Mosquito Repellent Patches</t>
         </is>
       </c>
       <c r="D915" s="2" t="n">
@@ -26098,7 +26098,7 @@
         </is>
       </c>
       <c r="D920" s="2" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E920" s="3" t="n">
         <v>13734</v>
@@ -26154,7 +26154,7 @@
         </is>
       </c>
       <c r="D922" s="2" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E922" s="3" t="n">
         <v>18059</v>
@@ -26182,7 +26182,7 @@
         </is>
       </c>
       <c r="D923" s="2" t="n">
-        <v>1792</v>
+        <v>1791</v>
       </c>
       <c r="E923" s="3" t="n">
         <v>3800</v>
@@ -26238,7 +26238,7 @@
         </is>
       </c>
       <c r="D925" s="2" t="n">
-        <v>1359</v>
+        <v>1345</v>
       </c>
       <c r="E925" s="3" t="n">
         <v>1195</v>
@@ -32538,7 +32538,7 @@
         </is>
       </c>
       <c r="D1150" s="2" t="n">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="E1150" s="3" t="n">
         <v>22558</v>
@@ -32707,7 +32707,7 @@
         </is>
       </c>
       <c r="D1156" s="2" t="n">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="E1156" s="3" t="n">
         <v>2338</v>
@@ -32763,7 +32763,7 @@
         </is>
       </c>
       <c r="D1158" s="2" t="n">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="E1158" s="3" t="n">
         <v>6039</v>
@@ -34499,7 +34499,7 @@
         </is>
       </c>
       <c r="D1220" s="2" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E1220" s="3" t="n">
         <v>37512</v>
@@ -36263,7 +36263,7 @@
         </is>
       </c>
       <c r="D1283" s="2" t="n">
-        <v>-3</v>
+        <v>21</v>
       </c>
       <c r="E1283" s="3" t="n">
         <v>5799</v>
@@ -45755,7 +45755,7 @@
         </is>
       </c>
       <c r="D1622" s="2" t="n">
-        <v>445</v>
+        <v>443</v>
       </c>
       <c r="E1622" s="3" t="n">
         <v>11372</v>
@@ -46399,7 +46399,7 @@
         </is>
       </c>
       <c r="D1645" s="2" t="n">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E1645" s="3" t="n">
         <v>16020</v>

</xml_diff>